<commit_message>
Flujo optimizado con validaciones y iteraciones entre registros solo exonerando a los que no alcanzaron cupo en los horarios establecidos
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -640,7 +640,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Error en procesamiento: No se encontró Nro Solicitud con token '29042'. Opciones: ['Seleccione']</t>
+          <t>No se encontró Nro Solicitud/Código de pago para token de 029042-0</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Error en procesamiento: No se encontró Nro Solicitud con token '29042'. Opciones: ['Seleccione']</t>
+          <t>No se encontró Nro Solicitud/Código de pago para token de 029042-0</t>
         </is>
       </c>
     </row>
@@ -785,6 +785,78 @@
       <c r="N5" t="inlineStr">
         <is>
           <t>No alcanzo cupo para horario 12:30-12:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>J &amp; V Resguardo</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>JEFATURA ZONAL DE JUNIN</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>31/03/26</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>12:30-12:45</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>25/03/2026</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>RENOVACIÓN DE LICENCIA DE USO</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>76734585</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>052340-0</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>CORTA</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>REVOLVER</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Documento vigilante no disponible para esta razón social/RUC. DNI=76734585 | RUC=J &amp; V Resguardo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Flujo conforme con iteraciones validadas y mostrado a Diana
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,27 +513,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>JEFATURA ZONAL LAMBAYEQUE (EX-INTENDENCIA II NORTE)</t>
+          <t>JEFATURA ZONAL DE ICA</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>07/04/26</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>10:30-10:45</t>
+          <t>09:00-09:15</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>25/03/2026</t>
+          <t>26/03/2026</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -543,12 +543,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>77276891</t>
+          <t>22100108</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>090086-0</t>
+          <t>079382-0</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -563,300 +563,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Cita Programada</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>No alcanzo cupo para horario 10:30-10:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>J &amp; V Resguardo</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>JEFATURA ZONAL DE JUNIN</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>31/03/2026</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>10:00-10:15</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>25/03/2026</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>INICIAL DE LICENCIA DE USO</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>46724112</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>029042-0</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>CORTA</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>REVOLVER</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>No se encontró Nro Solicitud/Código de pago para token de 029042-0</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>J &amp; V Resguardo</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>JEFATURA ZONAL DE JUNIN</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>31/03/2026</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>10:00-10:15</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>25/03/2026</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>INICIAL DE LICENCIA DE USO</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>46724112</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>029042-0</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>LARGA</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>ESCOPETA</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>No se encontró Nro Solicitud/Código de pago para token de 029042-0</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>J &amp; V Resguardo</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>LIMA</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>31/03/26</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>12:30-12:45</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>25/03/2026</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>RENOVACIÓN DE LICENCIA DE USO</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>44136452</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>052340-0</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>CORTA</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>REVOLVER</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>No alcanzo cupo para horario 12:30-12:45</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>J &amp; V Resguardo</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>JEFATURA ZONAL DE JUNIN</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>31/03/26</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>12:30-12:45</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>25/03/2026</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>RENOVACIÓN DE LICENCIA DE USO</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>76734585</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>052340-0</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>CORTA</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>REVOLVER</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Documento vigilante no disponible para esta razón social/RUC. DNI=76734585 | RUC=J &amp; V Resguardo</t>
+          <t>Error no mapeado persistente tras 4 intentos (hora=09:00-09:15, token=079382-0): No se pudo generar cita tras reintentos rápidos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Flujo pulido con validaciones y restricciones estrictas, así mismo con ruta ajustada solo para tolerar una única carpeta -ARMAS-GADSO-1.0-
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>30/03/2026</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>30/03/2026</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>30/03/2026</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Error no mapeado persistente tras 4 intentos (hora=10:45-11:00, token=049543-0): No se pudo confirmar la generación de cita de forma robusta (sin seales claras de xito y sin captcha incorrecto explícito)</t>
+          <t>No alcanzo cupo para horario 10:30-10:45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Flujo con multihilos implementado y respeta la logica inicial
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -566,9 +566,91 @@
         <v>Pendiente_x000d_</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>J &amp; V Resguardo</v>
+      </c>
+      <c r="C5" t="str">
+        <v>normal</v>
+      </c>
+      <c r="D5" t="str">
+        <v>JEFATURA ZONAL DE CAJAMARCA</v>
+      </c>
+      <c r="E5" t="str">
+        <v>31/03/2026</v>
+      </c>
+      <c r="F5" t="str">
+        <v>12:00-12:15</v>
+      </c>
+      <c r="G5" t="str">
+        <v>30/03/2026</v>
+      </c>
+      <c r="H5" t="str">
+        <v>RENOVACIÓN DE LICENCIA DE USO</v>
+      </c>
+      <c r="I5" t="str">
+        <v>09703265</v>
+      </c>
+      <c r="J5" t="str">
+        <v>038324-0</v>
+      </c>
+      <c r="K5" t="str">
+        <v>CORTA</v>
+      </c>
+      <c r="L5" t="str">
+        <v>PISTOLA</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Pendiente_x000d_</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>J &amp; V Resguardo</v>
+      </c>
+      <c r="C6" t="str">
+        <v>normal</v>
+      </c>
+      <c r="D6" t="str">
+        <v>JEFATURA ZONAL DE LA LIBERTAD</v>
+      </c>
+      <c r="E6" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="F6" t="str">
+        <v>09:45-10:00</v>
+      </c>
+      <c r="G6" t="str">
+        <v>30/03/2026</v>
+      </c>
+      <c r="H6" t="str">
+        <v>INICIAL DE LICENCIA DE USO</v>
+      </c>
+      <c r="I6" t="str">
+        <v>09703267</v>
+      </c>
+      <c r="J6" t="str">
+        <v>049543-0</v>
+      </c>
+      <c r="K6" t="str">
+        <v>CORTA</v>
+      </c>
+      <c r="L6" t="str">
+        <v>PISTOLA</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Pendiente_x000d_</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Flujo valido con hilos sin pertenecer a la estructura principal del flujo
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -454,31 +454,31 @@
         <v>normal</v>
       </c>
       <c r="D2" t="str">
-        <v>JEFATURA ZONAL DE LA LIBERTAD</v>
+        <v>LIMA</v>
       </c>
       <c r="E2" t="str">
-        <v>09/04/2026</v>
+        <v>21/04/2026</v>
       </c>
       <c r="F2" t="str">
-        <v>09:45-10:00</v>
+        <v>08:30-08:45</v>
       </c>
       <c r="G2" t="str">
-        <v>30/03/2026</v>
+        <v>31/03/2026</v>
       </c>
       <c r="H2" t="str">
         <v>INICIAL DE LICENCIA DE USO</v>
       </c>
       <c r="I2" t="str">
-        <v>09703265</v>
+        <v>77095597</v>
       </c>
       <c r="J2" t="str">
-        <v>049543-0</v>
+        <v>043788-0</v>
       </c>
       <c r="K2" t="str">
         <v>CORTA</v>
       </c>
       <c r="L2" t="str">
-        <v>PISTOLA</v>
+        <v>REVOLVER</v>
       </c>
       <c r="M2" t="str">
         <v>Pendiente_x000d_</v>
@@ -495,25 +495,25 @@
         <v>normal</v>
       </c>
       <c r="D3" t="str">
-        <v>JEFATURA ZONAL DE TACNA</v>
+        <v>LIMA</v>
       </c>
       <c r="E3" t="str">
+        <v>21/04/2026</v>
+      </c>
+      <c r="F3" t="str">
+        <v>09:00-09:15</v>
+      </c>
+      <c r="G3" t="str">
         <v>31/03/2026</v>
-      </c>
-      <c r="F3" t="str">
-        <v>12:15-12:30</v>
-      </c>
-      <c r="G3" t="str">
-        <v>30/03/2026</v>
       </c>
       <c r="H3" t="str">
         <v>RENOVACIÓN DE LICENCIA DE USO</v>
       </c>
       <c r="I3" t="str">
-        <v>10595436</v>
+        <v>08666044</v>
       </c>
       <c r="J3" t="str">
-        <v>052335-0</v>
+        <v>043503-0</v>
       </c>
       <c r="K3" t="str">
         <v>CORTA</v>
@@ -536,25 +536,25 @@
         <v>normal</v>
       </c>
       <c r="D4" t="str">
-        <v>JEFATURA ZONAL AREQUIPA (EX-INTENDENCIA III SUR)</v>
+        <v>LIMA</v>
       </c>
       <c r="E4" t="str">
+        <v>21/04/2026</v>
+      </c>
+      <c r="F4" t="str">
+        <v>09:00-09:15</v>
+      </c>
+      <c r="G4" t="str">
         <v>31/03/2026</v>
-      </c>
-      <c r="F4" t="str">
-        <v>08:45-09:00</v>
-      </c>
-      <c r="G4" t="str">
-        <v>30/03/2026</v>
       </c>
       <c r="H4" t="str">
         <v>RENOVACIÓN DE LICENCIA DE USO</v>
       </c>
       <c r="I4" t="str">
-        <v>09703265</v>
+        <v>15740016</v>
       </c>
       <c r="J4" t="str">
-        <v>075373-0</v>
+        <v>043504-0</v>
       </c>
       <c r="K4" t="str">
         <v>CORTA</v>
@@ -568,89 +568,12 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>4</v>
-      </c>
-      <c r="B5" t="str">
-        <v>J &amp; V Resguardo</v>
-      </c>
-      <c r="C5" t="str">
-        <v>normal</v>
-      </c>
-      <c r="D5" t="str">
-        <v>JEFATURA ZONAL DE CAJAMARCA</v>
-      </c>
-      <c r="E5" t="str">
-        <v>31/03/2026</v>
-      </c>
-      <c r="F5" t="str">
-        <v>12:00-12:15</v>
-      </c>
-      <c r="G5" t="str">
-        <v>30/03/2026</v>
-      </c>
-      <c r="H5" t="str">
-        <v>RENOVACIÓN DE LICENCIA DE USO</v>
-      </c>
-      <c r="I5" t="str">
-        <v>09703265</v>
-      </c>
-      <c r="J5" t="str">
-        <v>038324-0</v>
-      </c>
-      <c r="K5" t="str">
-        <v>CORTA</v>
-      </c>
-      <c r="L5" t="str">
-        <v>PISTOLA</v>
-      </c>
-      <c r="M5" t="str">
-        <v>Pendiente_x000d_</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>J &amp; V Resguardo</v>
-      </c>
-      <c r="C6" t="str">
-        <v>normal</v>
-      </c>
-      <c r="D6" t="str">
-        <v>JEFATURA ZONAL DE LA LIBERTAD</v>
-      </c>
-      <c r="E6" t="str">
-        <v>09/04/2026</v>
-      </c>
-      <c r="F6" t="str">
-        <v>09:45-10:00</v>
-      </c>
-      <c r="G6" t="str">
-        <v>30/03/2026</v>
-      </c>
-      <c r="H6" t="str">
-        <v>INICIAL DE LICENCIA DE USO</v>
-      </c>
-      <c r="I6" t="str">
-        <v>09703267</v>
-      </c>
-      <c r="J6" t="str">
-        <v>049543-0</v>
-      </c>
-      <c r="K6" t="str">
-        <v>CORTA</v>
-      </c>
-      <c r="L6" t="str">
-        <v>PISTOLA</v>
-      </c>
-      <c r="M6" t="str">
-        <v>Pendiente_x000d_</v>
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Flujo con validación de id dinámico multihilo
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -451,28 +451,28 @@
         <v>J &amp; V Resguardo</v>
       </c>
       <c r="C2" t="str">
-        <v>normal</v>
+        <v>alta</v>
       </c>
       <c r="D2" t="str">
         <v>LIMA</v>
       </c>
       <c r="E2" t="str">
-        <v>21/04/2026</v>
+        <v>22/04/2026</v>
       </c>
       <c r="F2" t="str">
-        <v>08:30-08:45</v>
+        <v>08:00-08:15</v>
       </c>
       <c r="G2" t="str">
-        <v>31/03/2026</v>
+        <v>1/04/2026</v>
       </c>
       <c r="H2" t="str">
         <v>INICIAL DE LICENCIA DE USO</v>
       </c>
       <c r="I2" t="str">
-        <v>77095597</v>
+        <v>09452250</v>
       </c>
       <c r="J2" t="str">
-        <v>043788-0</v>
+        <v>080000-0</v>
       </c>
       <c r="K2" t="str">
         <v>CORTA</v>
@@ -492,28 +492,28 @@
         <v>J &amp; V Resguardo</v>
       </c>
       <c r="C3" t="str">
-        <v>normal</v>
+        <v>alta</v>
       </c>
       <c r="D3" t="str">
         <v>LIMA</v>
       </c>
       <c r="E3" t="str">
-        <v>21/04/2026</v>
+        <v>22/04/2026</v>
       </c>
       <c r="F3" t="str">
         <v>09:00-09:15</v>
       </c>
       <c r="G3" t="str">
-        <v>31/03/2026</v>
+        <v>1/04/2026</v>
       </c>
       <c r="H3" t="str">
         <v>RENOVACIÓN DE LICENCIA DE USO</v>
       </c>
       <c r="I3" t="str">
-        <v>08666044</v>
+        <v>43440164</v>
       </c>
       <c r="J3" t="str">
-        <v>043503-0</v>
+        <v>068399-0</v>
       </c>
       <c r="K3" t="str">
         <v>CORTA</v>
@@ -539,28 +539,28 @@
         <v>LIMA</v>
       </c>
       <c r="E4" t="str">
-        <v>21/04/2026</v>
+        <v>22/04/2026</v>
       </c>
       <c r="F4" t="str">
-        <v>09:00-09:15</v>
+        <v>08:00-08:15</v>
       </c>
       <c r="G4" t="str">
-        <v>31/03/2026</v>
+        <v>1/04/2026</v>
       </c>
       <c r="H4" t="str">
         <v>RENOVACIÓN DE LICENCIA DE USO</v>
       </c>
       <c r="I4" t="str">
-        <v>15740016</v>
+        <v>60274318</v>
       </c>
       <c r="J4" t="str">
-        <v>043504-0</v>
+        <v>094587-0</v>
       </c>
       <c r="K4" t="str">
         <v>CORTA</v>
       </c>
       <c r="L4" t="str">
-        <v>PISTOLA</v>
+        <v>REVOLVER</v>
       </c>
       <c r="M4" t="str">
         <v>Pendiente_x000d_</v>
@@ -568,12 +568,53 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>J &amp; V Resguardo</v>
+      </c>
+      <c r="C5" t="str">
+        <v>normal</v>
+      </c>
+      <c r="D5" t="str">
+        <v>LIMA</v>
+      </c>
+      <c r="E5" t="str">
+        <v>22/04/2026</v>
+      </c>
+      <c r="F5" t="str">
+        <v>09:00-09:15</v>
+      </c>
+      <c r="G5" t="str">
+        <v>1/04/2026</v>
+      </c>
+      <c r="H5" t="str">
+        <v>RENOVACIÓN DE LICENCIA DE USO</v>
+      </c>
+      <c r="I5" t="str">
+        <v>75151780</v>
+      </c>
+      <c r="J5" t="str">
+        <v>052332-0</v>
+      </c>
+      <c r="K5" t="str">
+        <v>CORTA</v>
+      </c>
+      <c r="L5" t="str">
+        <v>REVOLVER</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Pendiente_x000d_</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Solución de error con botón Generar Cita Hardcordeado
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -457,22 +457,22 @@
         <v>LIMA</v>
       </c>
       <c r="E2" t="str">
-        <v>7/05/2026</v>
+        <v>8/05/2026</v>
       </c>
       <c r="F2" t="str">
         <v>12:00-12:15</v>
       </c>
       <c r="G2" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="H2" t="str">
-        <v>RENOVACION DE LICENCIA DE USO</v>
+        <v>INICIAL DE LICENCIA DE USO</v>
       </c>
       <c r="I2" t="str">
-        <v>45429407</v>
+        <v>76023039</v>
       </c>
       <c r="J2" t="str">
-        <v>098411-0</v>
+        <v>043793-0</v>
       </c>
       <c r="K2" t="str">
         <v>CORTA</v>
@@ -498,22 +498,22 @@
         <v>LIMA</v>
       </c>
       <c r="E3" t="str">
-        <v>7/05/2026</v>
+        <v>8/05/2026</v>
       </c>
       <c r="F3" t="str">
-        <v>12:15-12:30</v>
+        <v>12:00-12:15</v>
       </c>
       <c r="G3" t="str">
-        <v>16/04/2026</v>
+        <v>17/04/2026</v>
       </c>
       <c r="H3" t="str">
-        <v>INICIAL DE LICENCIA DE USO</v>
+        <v>RENOVACION DE LICENCIA DE USO</v>
       </c>
       <c r="I3" t="str">
-        <v>10212773</v>
+        <v>00966547</v>
       </c>
       <c r="J3" t="str">
-        <v>071549-0</v>
+        <v>098412-0</v>
       </c>
       <c r="K3" t="str">
         <v>CORTA</v>
@@ -523,6 +523,52 @@
       </c>
       <c r="M3" t="str">
         <v>Pendiente_x000d_</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>J &amp; V Resguardo</v>
+      </c>
+      <c r="C4" t="str">
+        <v>alta</v>
+      </c>
+      <c r="D4" t="str">
+        <v>LIMA</v>
+      </c>
+      <c r="E4" t="str">
+        <v>8/05/2026</v>
+      </c>
+      <c r="F4" t="str">
+        <v>11:45-12:00</v>
+      </c>
+      <c r="G4" t="str">
+        <v>17/04/2026</v>
+      </c>
+      <c r="H4" t="str">
+        <v>RENOVACION DE LICENCIA DE USO</v>
+      </c>
+      <c r="I4" t="str">
+        <v>45759844</v>
+      </c>
+      <c r="J4" t="str">
+        <v>085709-0</v>
+      </c>
+      <c r="K4" t="str">
+        <v>CORTA</v>
+      </c>
+      <c r="L4" t="str">
+        <v>PISTOLA</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Pendiente_x000d_</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Flujo con pequeñas validaciones y capturas, previas a refactorizar toda la arquitectura
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -457,13 +457,13 @@
         <v>LIMA</v>
       </c>
       <c r="E2" t="str">
-        <v>8/05/2026</v>
+        <v>15/05/2026</v>
       </c>
       <c r="F2" t="str">
         <v>12:00-12:15</v>
       </c>
       <c r="G2" t="str">
-        <v>17/04/2026</v>
+        <v>24/04/2026</v>
       </c>
       <c r="H2" t="str">
         <v>INICIAL DE LICENCIA DE USO</v>
@@ -498,22 +498,22 @@
         <v>LIMA</v>
       </c>
       <c r="E3" t="str">
-        <v>8/05/2026</v>
+        <v>15/05/2026</v>
       </c>
       <c r="F3" t="str">
         <v>12:00-12:15</v>
       </c>
       <c r="G3" t="str">
-        <v>17/04/2026</v>
+        <v>24/04/2026</v>
       </c>
       <c r="H3" t="str">
-        <v>RENOVACION DE LICENCIA DE USO</v>
+        <v>RENOVACIÓN DE LICENCIA DE USO</v>
       </c>
       <c r="I3" t="str">
-        <v>00966547</v>
+        <v>47694399</v>
       </c>
       <c r="J3" t="str">
-        <v>098412-0</v>
+        <v>099008-0</v>
       </c>
       <c r="K3" t="str">
         <v>CORTA</v>
@@ -527,47 +527,6 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>J &amp; V Resguardo</v>
-      </c>
-      <c r="C4" t="str">
-        <v>alta</v>
-      </c>
-      <c r="D4" t="str">
-        <v>LIMA</v>
-      </c>
-      <c r="E4" t="str">
-        <v>8/05/2026</v>
-      </c>
-      <c r="F4" t="str">
-        <v>11:45-12:00</v>
-      </c>
-      <c r="G4" t="str">
-        <v>17/04/2026</v>
-      </c>
-      <c r="H4" t="str">
-        <v>RENOVACION DE LICENCIA DE USO</v>
-      </c>
-      <c r="I4" t="str">
-        <v>45759844</v>
-      </c>
-      <c r="J4" t="str">
-        <v>085709-0</v>
-      </c>
-      <c r="K4" t="str">
-        <v>CORTA</v>
-      </c>
-      <c r="L4" t="str">
-        <v>PISTOLA</v>
-      </c>
-      <c r="M4" t="str">
-        <v>Pendiente_x000d_</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
         <v/>
       </c>
     </row>
@@ -576,9 +535,14 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Flujo refactorizado, con arquitectura limpia, validaciones estrictas y dependencias segmentadas por etapa del flujo
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -454,25 +454,25 @@
         <v>alta</v>
       </c>
       <c r="D2" t="str">
-        <v>LIMA</v>
+        <v>JEFATURA ZONAL DE ICA</v>
       </c>
       <c r="E2" t="str">
-        <v>15/05/2026</v>
+        <v>30/04/2026</v>
       </c>
       <c r="F2" t="str">
-        <v>12:00-12:15</v>
+        <v>10:00-10:15</v>
       </c>
       <c r="G2" t="str">
         <v>24/04/2026</v>
       </c>
       <c r="H2" t="str">
-        <v>INICIAL DE LICENCIA DE USO</v>
+        <v>RENOVACION DE LICENCIA DE USO</v>
       </c>
       <c r="I2" t="str">
-        <v>76023039</v>
+        <v>60389562</v>
       </c>
       <c r="J2" t="str">
-        <v>043793-0</v>
+        <v>085704-0</v>
       </c>
       <c r="K2" t="str">
         <v>CORTA</v>
@@ -481,47 +481,6 @@
         <v>REVOLVER</v>
       </c>
       <c r="M2" t="str">
-        <v>Pendiente_x000d_</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>J &amp; V Resguardo</v>
-      </c>
-      <c r="C3" t="str">
-        <v>alta</v>
-      </c>
-      <c r="D3" t="str">
-        <v>LIMA</v>
-      </c>
-      <c r="E3" t="str">
-        <v>15/05/2026</v>
-      </c>
-      <c r="F3" t="str">
-        <v>12:00-12:15</v>
-      </c>
-      <c r="G3" t="str">
-        <v>24/04/2026</v>
-      </c>
-      <c r="H3" t="str">
-        <v>RENOVACIÓN DE LICENCIA DE USO</v>
-      </c>
-      <c r="I3" t="str">
-        <v>47694399</v>
-      </c>
-      <c r="J3" t="str">
-        <v>099008-0</v>
-      </c>
-      <c r="K3" t="str">
-        <v>CORTA</v>
-      </c>
-      <c r="L3" t="str">
-        <v>REVOLVER</v>
-      </c>
-      <c r="M3" t="str">
         <v>Pendiente_x000d_</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ingregación de envío de correos con API Microsoft Grafh
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -454,25 +454,25 @@
         <v>alta</v>
       </c>
       <c r="D2" t="str">
-        <v>JEFATURA ZONAL DE ICA</v>
+        <v>LIMA</v>
       </c>
       <c r="E2" t="str">
-        <v>30/04/2026</v>
+        <v>19/05/2026</v>
       </c>
       <c r="F2" t="str">
-        <v>10:00-10:15</v>
+        <v>12:00-12:15</v>
       </c>
       <c r="G2" t="str">
-        <v>24/04/2026</v>
+        <v>28/04/2026</v>
       </c>
       <c r="H2" t="str">
         <v>RENOVACION DE LICENCIA DE USO</v>
       </c>
       <c r="I2" t="str">
-        <v>60389562</v>
+        <v>40598949</v>
       </c>
       <c r="J2" t="str">
-        <v>085704-0</v>
+        <v>052333-0</v>
       </c>
       <c r="K2" t="str">
         <v>CORTA</v>
@@ -481,6 +481,47 @@
         <v>REVOLVER</v>
       </c>
       <c r="M2" t="str">
+        <v>Pendiente_x000d_</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>J &amp; V Resguardo</v>
+      </c>
+      <c r="C3" t="str">
+        <v>alta</v>
+      </c>
+      <c r="D3" t="str">
+        <v>LIMA</v>
+      </c>
+      <c r="E3" t="str">
+        <v>19/05/2026</v>
+      </c>
+      <c r="F3" t="str">
+        <v>12:00-12:15</v>
+      </c>
+      <c r="G3" t="str">
+        <v>28/04/2026</v>
+      </c>
+      <c r="H3" t="str">
+        <v>RENOVACION DE LICENCIA DE USO</v>
+      </c>
+      <c r="I3" t="str">
+        <v>73799884</v>
+      </c>
+      <c r="J3" t="str">
+        <v>037411-0</v>
+      </c>
+      <c r="K3" t="str">
+        <v>CORTA</v>
+      </c>
+      <c r="L3" t="str">
+        <v>REVOLVER</v>
+      </c>
+      <c r="M3" t="str">
         <v>Pendiente_x000d_</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactorizaciones: Nuevo error curs 48h + logs de correo
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -457,28 +457,28 @@
         <v>LIMA</v>
       </c>
       <c r="E2" t="str">
-        <v>19/05/2026</v>
+        <v>29/05/2026</v>
       </c>
       <c r="F2" t="str">
-        <v>12:00-12:15</v>
+        <v>08:00-08:15</v>
       </c>
       <c r="G2" t="str">
-        <v>28/04/2026</v>
+        <v>8/05/2026</v>
       </c>
       <c r="H2" t="str">
         <v>RENOVACION DE LICENCIA DE USO</v>
       </c>
       <c r="I2" t="str">
-        <v>40598949</v>
+        <v>09627091</v>
       </c>
       <c r="J2" t="str">
-        <v>052333-0</v>
+        <v>060579-0</v>
       </c>
       <c r="K2" t="str">
         <v>CORTA</v>
       </c>
       <c r="L2" t="str">
-        <v>REVOLVER</v>
+        <v>PISTOLA</v>
       </c>
       <c r="M2" t="str">
         <v>Pendiente_x000d_</v>
@@ -498,28 +498,28 @@
         <v>LIMA</v>
       </c>
       <c r="E3" t="str">
-        <v>19/05/2026</v>
+        <v>29/05/2026</v>
       </c>
       <c r="F3" t="str">
-        <v>12:00-12:15</v>
+        <v>08:15-08:30</v>
       </c>
       <c r="G3" t="str">
-        <v>28/04/2026</v>
+        <v>8/05/2026</v>
       </c>
       <c r="H3" t="str">
         <v>RENOVACION DE LICENCIA DE USO</v>
       </c>
       <c r="I3" t="str">
-        <v>73799884</v>
+        <v>10198664</v>
       </c>
       <c r="J3" t="str">
-        <v>037411-0</v>
+        <v>020858-0</v>
       </c>
       <c r="K3" t="str">
         <v>CORTA</v>
       </c>
       <c r="L3" t="str">
-        <v>REVOLVER</v>
+        <v>PISTOLA</v>
       </c>
       <c r="M3" t="str">
         <v>Pendiente_x000d_</v>
@@ -527,22 +527,258 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>J &amp; V Resguardo</v>
+      </c>
+      <c r="C4" t="str">
+        <v>alta</v>
+      </c>
+      <c r="D4" t="str">
+        <v>LIMA</v>
+      </c>
+      <c r="E4" t="str">
+        <v>29/05/2026</v>
+      </c>
+      <c r="F4" t="str">
+        <v>09:00-09:15</v>
+      </c>
+      <c r="G4" t="str">
+        <v>8/05/2026</v>
+      </c>
+      <c r="H4" t="str">
+        <v>RENOVACION DE LICENCIA DE USO</v>
+      </c>
+      <c r="I4" t="str">
+        <v>10439677</v>
+      </c>
+      <c r="J4" t="str">
+        <v>099009-0</v>
+      </c>
+      <c r="K4" t="str">
+        <v>CORTA</v>
+      </c>
+      <c r="L4" t="str">
+        <v>REVOLVER</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Pendiente_x000d_</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>J &amp; V Resguardo</v>
+      </c>
+      <c r="C5" t="str">
+        <v>alta</v>
+      </c>
+      <c r="D5" t="str">
+        <v>LIMA</v>
+      </c>
+      <c r="E5" t="str">
+        <v>29/05/2026</v>
+      </c>
+      <c r="F5" t="str">
+        <v>11:15-11:30</v>
+      </c>
+      <c r="G5" t="str">
+        <v>8/05/2026</v>
+      </c>
+      <c r="H5" t="str">
+        <v>INICIAL DE LICENCIA DE USO</v>
+      </c>
+      <c r="I5" t="str">
+        <v>78997430</v>
+      </c>
+      <c r="J5" t="str">
+        <v>100403-0</v>
+      </c>
+      <c r="K5" t="str">
+        <v>CORTA</v>
+      </c>
+      <c r="L5" t="str">
+        <v>REVOLVER</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Pendiente_x000d_</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>J &amp; V Resguardo</v>
+      </c>
+      <c r="C6" t="str">
+        <v>alta</v>
+      </c>
+      <c r="D6" t="str">
+        <v>LIMA</v>
+      </c>
+      <c r="E6" t="str">
+        <v>29/05/2026</v>
+      </c>
+      <c r="F6" t="str">
+        <v>11:15-11:30</v>
+      </c>
+      <c r="G6" t="str">
+        <v>8/05/2026</v>
+      </c>
+      <c r="H6" t="str">
+        <v>INICIAL DE LICENCIA DE USO</v>
+      </c>
+      <c r="I6" t="str">
+        <v>78997430</v>
+      </c>
+      <c r="J6" t="str">
+        <v>100403-0</v>
+      </c>
+      <c r="K6" t="str">
+        <v>LARGA</v>
+      </c>
+      <c r="L6" t="str">
+        <v>ESCOPETA</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Pendiente_x000d_</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>J &amp; V Resguardo</v>
+      </c>
+      <c r="C7" t="str">
+        <v>alta</v>
+      </c>
+      <c r="D7" t="str">
+        <v>LIMA</v>
+      </c>
+      <c r="E7" t="str">
+        <v>29/05/2026</v>
+      </c>
+      <c r="F7" t="str">
+        <v>11:30-11:45</v>
+      </c>
+      <c r="G7" t="str">
+        <v>8/05/2026</v>
+      </c>
+      <c r="H7" t="str">
+        <v>INICIAL DE LICENCIA DE USO</v>
+      </c>
+      <c r="I7" t="str">
+        <v>76477494</v>
+      </c>
+      <c r="J7" t="str">
+        <v xml:space="preserve">052418-0 </v>
+      </c>
+      <c r="K7" t="str">
+        <v>CORTA</v>
+      </c>
+      <c r="L7" t="str">
+        <v>REVOLVER</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Pendiente_x000d_</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>J &amp; V Resguardo</v>
+      </c>
+      <c r="C8" t="str">
+        <v>alta</v>
+      </c>
+      <c r="D8" t="str">
+        <v>LIMA</v>
+      </c>
+      <c r="E8" t="str">
+        <v>29/05/2026</v>
+      </c>
+      <c r="F8" t="str">
+        <v>11:30-11:45</v>
+      </c>
+      <c r="G8" t="str">
+        <v>8/05/2026</v>
+      </c>
+      <c r="H8" t="str">
+        <v>INICIAL DE LICENCIA DE USO</v>
+      </c>
+      <c r="I8" t="str">
+        <v>76477494</v>
+      </c>
+      <c r="J8" t="str">
+        <v xml:space="preserve">052418-0 </v>
+      </c>
+      <c r="K8" t="str">
+        <v>LARGA</v>
+      </c>
+      <c r="L8" t="str">
+        <v>ESCOPETA</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Pendiente_x000d_</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>J &amp; V Resguardo</v>
+      </c>
+      <c r="C9" t="str">
+        <v>alta</v>
+      </c>
+      <c r="D9" t="str">
+        <v>LIMA</v>
+      </c>
+      <c r="E9" t="str">
+        <v>29/05/2026</v>
+      </c>
+      <c r="F9" t="str">
+        <v>12:00-12:15</v>
+      </c>
+      <c r="G9" t="str">
+        <v>8/05/2026</v>
+      </c>
+      <c r="H9" t="str">
+        <v>RENOVACION DE LICENCIA DE USO</v>
+      </c>
+      <c r="I9" t="str">
+        <v>00966547</v>
+      </c>
+      <c r="J9" t="str">
+        <v>098412-0</v>
+      </c>
+      <c r="K9" t="str">
+        <v>CORTA</v>
+      </c>
+      <c r="L9" t="str">
+        <v>REVOLVER</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Pendiente_x000d_</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
REFACTOR: Consistencia de elementos
</commit_message>
<xml_diff>
--- a/data/programaciones-armas.xlsx
+++ b/data/programaciones-armas.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -457,28 +457,28 @@
         <v>LIMA</v>
       </c>
       <c r="E2" t="str">
-        <v>29/05/2026</v>
+        <v>11/06/2026</v>
       </c>
       <c r="F2" t="str">
-        <v>08:00-08:15</v>
+        <v>12:30-12:45</v>
       </c>
       <c r="G2" t="str">
-        <v>8/05/2026</v>
+        <v>21/05/2026</v>
       </c>
       <c r="H2" t="str">
         <v>RENOVACION DE LICENCIA DE USO</v>
       </c>
       <c r="I2" t="str">
-        <v>09627091</v>
+        <v>77276891</v>
       </c>
       <c r="J2" t="str">
-        <v>060579-0</v>
+        <v>034550-0</v>
       </c>
       <c r="K2" t="str">
         <v>CORTA</v>
       </c>
       <c r="L2" t="str">
-        <v>PISTOLA</v>
+        <v>REVOLVER</v>
       </c>
       <c r="M2" t="str">
         <v>Pendiente_x000d_</v>
@@ -486,7 +486,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="str">
         <v>J &amp; V Resguardo</v>
@@ -498,28 +498,28 @@
         <v>LIMA</v>
       </c>
       <c r="E3" t="str">
-        <v>29/05/2026</v>
+        <v>11/06/2026</v>
       </c>
       <c r="F3" t="str">
-        <v>08:15-08:30</v>
+        <v>12:30-12:45</v>
       </c>
       <c r="G3" t="str">
-        <v>8/05/2026</v>
+        <v>21/05/2026</v>
       </c>
       <c r="H3" t="str">
         <v>RENOVACION DE LICENCIA DE USO</v>
       </c>
       <c r="I3" t="str">
-        <v>10198664</v>
+        <v>77276891</v>
       </c>
       <c r="J3" t="str">
-        <v>020858-0</v>
+        <v>034550-0</v>
       </c>
       <c r="K3" t="str">
-        <v>CORTA</v>
+        <v>LARGA</v>
       </c>
       <c r="L3" t="str">
-        <v>PISTOLA</v>
+        <v>ESCOPETA</v>
       </c>
       <c r="M3" t="str">
         <v>Pendiente_x000d_</v>
@@ -527,7 +527,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" t="str">
         <v>J &amp; V Resguardo</v>
@@ -539,22 +539,22 @@
         <v>LIMA</v>
       </c>
       <c r="E4" t="str">
-        <v>29/05/2026</v>
+        <v>11/06/2026</v>
       </c>
       <c r="F4" t="str">
-        <v>09:00-09:15</v>
+        <v>12:30-12:45</v>
       </c>
       <c r="G4" t="str">
-        <v>8/05/2026</v>
+        <v>21/05/2026</v>
       </c>
       <c r="H4" t="str">
         <v>RENOVACION DE LICENCIA DE USO</v>
       </c>
       <c r="I4" t="str">
-        <v>10439677</v>
+        <v>74388142</v>
       </c>
       <c r="J4" t="str">
-        <v>099009-0</v>
+        <v>028816-0</v>
       </c>
       <c r="K4" t="str">
         <v>CORTA</v>
@@ -568,7 +568,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" t="str">
         <v>J &amp; V Resguardo</v>
@@ -580,22 +580,22 @@
         <v>LIMA</v>
       </c>
       <c r="E5" t="str">
-        <v>29/05/2026</v>
+        <v>11/06/2026</v>
       </c>
       <c r="F5" t="str">
-        <v>11:15-11:30</v>
+        <v>12:15-12:30</v>
       </c>
       <c r="G5" t="str">
-        <v>8/05/2026</v>
+        <v>21/05/2026</v>
       </c>
       <c r="H5" t="str">
-        <v>INICIAL DE LICENCIA DE USO</v>
+        <v>RENOVACION DE LICENCIA DE USO</v>
       </c>
       <c r="I5" t="str">
-        <v>78997430</v>
+        <v>62160619</v>
       </c>
       <c r="J5" t="str">
-        <v>100403-0</v>
+        <v>028818-0</v>
       </c>
       <c r="K5" t="str">
         <v>CORTA</v>
@@ -609,7 +609,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B6" t="str">
         <v>J &amp; V Resguardo</v>
@@ -621,22 +621,22 @@
         <v>LIMA</v>
       </c>
       <c r="E6" t="str">
-        <v>29/05/2026</v>
+        <v>11/06/2026</v>
       </c>
       <c r="F6" t="str">
-        <v>11:15-11:30</v>
+        <v>12:15-12:30</v>
       </c>
       <c r="G6" t="str">
-        <v>8/05/2026</v>
+        <v>21/05/2026</v>
       </c>
       <c r="H6" t="str">
-        <v>INICIAL DE LICENCIA DE USO</v>
+        <v>RENOVACION DE LICENCIA DE USO</v>
       </c>
       <c r="I6" t="str">
-        <v>78997430</v>
+        <v>62160619</v>
       </c>
       <c r="J6" t="str">
-        <v>100403-0</v>
+        <v>028818-0</v>
       </c>
       <c r="K6" t="str">
         <v>LARGA</v>
@@ -650,7 +650,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B7" t="str">
         <v>J &amp; V Resguardo</v>
@@ -662,22 +662,22 @@
         <v>LIMA</v>
       </c>
       <c r="E7" t="str">
-        <v>29/05/2026</v>
+        <v>11/06/2026</v>
       </c>
       <c r="F7" t="str">
-        <v>11:30-11:45</v>
+        <v>12:00-12:15</v>
       </c>
       <c r="G7" t="str">
-        <v>8/05/2026</v>
+        <v>21/05/2026</v>
       </c>
       <c r="H7" t="str">
-        <v>INICIAL DE LICENCIA DE USO</v>
+        <v>RENOVACION DE LICENCIA DE USO</v>
       </c>
       <c r="I7" t="str">
-        <v>76477494</v>
+        <v>43507007</v>
       </c>
       <c r="J7" t="str">
-        <v xml:space="preserve">052418-0 </v>
+        <v>008895-0</v>
       </c>
       <c r="K7" t="str">
         <v>CORTA</v>
@@ -691,7 +691,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B8" t="str">
         <v>J &amp; V Resguardo</v>
@@ -703,22 +703,22 @@
         <v>LIMA</v>
       </c>
       <c r="E8" t="str">
-        <v>29/05/2026</v>
+        <v>11/06/2026</v>
       </c>
       <c r="F8" t="str">
-        <v>11:30-11:45</v>
+        <v>12:00-12:15</v>
       </c>
       <c r="G8" t="str">
-        <v>8/05/2026</v>
+        <v>21/05/2026</v>
       </c>
       <c r="H8" t="str">
-        <v>INICIAL DE LICENCIA DE USO</v>
+        <v>RENOVACION DE LICENCIA DE USO</v>
       </c>
       <c r="I8" t="str">
-        <v>76477494</v>
+        <v>43507007</v>
       </c>
       <c r="J8" t="str">
-        <v xml:space="preserve">052418-0 </v>
+        <v>008895-0</v>
       </c>
       <c r="K8" t="str">
         <v>LARGA</v>
@@ -732,7 +732,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B9" t="str">
         <v>J &amp; V Resguardo</v>
@@ -744,22 +744,22 @@
         <v>LIMA</v>
       </c>
       <c r="E9" t="str">
-        <v>29/05/2026</v>
+        <v>11/06/2026</v>
       </c>
       <c r="F9" t="str">
-        <v>12:00-12:15</v>
+        <v>12:15-12:30</v>
       </c>
       <c r="G9" t="str">
-        <v>8/05/2026</v>
+        <v>21/05/2026</v>
       </c>
       <c r="H9" t="str">
         <v>RENOVACION DE LICENCIA DE USO</v>
       </c>
       <c r="I9" t="str">
-        <v>00966547</v>
+        <v>40016403</v>
       </c>
       <c r="J9" t="str">
-        <v>098412-0</v>
+        <v>008896-0</v>
       </c>
       <c r="K9" t="str">
         <v>CORTA</v>
@@ -773,12 +773,53 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>5</v>
+      </c>
+      <c r="B10" t="str">
+        <v>J &amp; V Resguardo</v>
+      </c>
+      <c r="C10" t="str">
+        <v>alta</v>
+      </c>
+      <c r="D10" t="str">
+        <v>LIMA</v>
+      </c>
+      <c r="E10" t="str">
+        <v>11/06/2026</v>
+      </c>
+      <c r="F10" t="str">
+        <v>12:15-12:30</v>
+      </c>
+      <c r="G10" t="str">
+        <v>21/05/2026</v>
+      </c>
+      <c r="H10" t="str">
+        <v>RENOVACION DE LICENCIA DE USO</v>
+      </c>
+      <c r="I10" t="str">
+        <v>40016403</v>
+      </c>
+      <c r="J10" t="str">
+        <v>008896-0</v>
+      </c>
+      <c r="K10" t="str">
+        <v>LARGA</v>
+      </c>
+      <c r="L10" t="str">
+        <v>ESCOPETA</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Pendiente_x000d_</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>